<commit_message>
Add manual testing documentation
</commit_message>
<xml_diff>
--- a/test_cases/SauceDemo QA Project.xlsx
+++ b/test_cases/SauceDemo QA Project.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Desktop\SauceDemo-Automation\test_cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F37FF4F6-89CA-4C55-8C9C-2B66D5300121}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="6" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1286,13 +1286,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1307,13 +1306,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1325,9 +1321,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1357,6 +1350,9 @@
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1654,31 +1650,31 @@
   </cols>
   <sheetData>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="G4" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="H4" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="I4" s="10" t="s">
+      <c r="I4" s="9" t="s">
         <v>24</v>
       </c>
     </row>
@@ -1709,7 +1705,7 @@
       <c r="E6" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="2" t="s">
         <v>33</v>
       </c>
       <c r="G6" s="2" t="s">
@@ -1790,10 +1786,10 @@
       <c r="E11" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="G11" s="3" t="s">
         <v>41</v>
       </c>
       <c r="H11" t="s">
@@ -1856,7 +1852,7 @@
       <c r="I15" s="2"/>
     </row>
     <row r="16" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A16" s="6" t="s">
+      <c r="A16" s="5" t="s">
         <v>5</v>
       </c>
       <c r="B16" t="s">
@@ -2074,17 +2070,17 @@
       <c r="I28" s="2"/>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A29" s="5"/>
-      <c r="B29" s="5"/>
-      <c r="C29" s="5"/>
+      <c r="A29" s="4"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
       <c r="D29" t="s">
         <v>29</v>
       </c>
-      <c r="E29" s="5"/>
-      <c r="F29" s="5"/>
-      <c r="G29" s="5"/>
-      <c r="H29" s="5"/>
-      <c r="I29" s="5"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4"/>
+      <c r="I29" s="4"/>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" s="2"/>
@@ -2283,7 +2279,7 @@
       <c r="D42" t="s">
         <v>26</v>
       </c>
-      <c r="E42" s="8"/>
+      <c r="E42" s="7"/>
       <c r="F42" t="s">
         <v>67</v>
       </c>
@@ -2304,7 +2300,7 @@
       <c r="D43" t="s">
         <v>64</v>
       </c>
-      <c r="E43" s="7" t="s">
+      <c r="E43" s="6" t="s">
         <v>30</v>
       </c>
       <c r="F43" s="2"/>
@@ -2645,250 +2641,250 @@
   </cols>
   <sheetData>
     <row r="3" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E3" s="24" t="s">
+      <c r="E3" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="F3" s="24" t="s">
+      <c r="F3" s="21" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="4" spans="5:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="E4" s="22" t="s">
+      <c r="E4" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="F4" s="22" t="s">
+      <c r="F4" s="19" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="5" spans="5:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="E5" s="22" t="s">
+      <c r="E5" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="F5" s="22" t="s">
+      <c r="F5" s="19" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="6" spans="5:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="E6" s="22" t="s">
+      <c r="E6" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="F6" s="22" t="s">
+      <c r="F6" s="19" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="7" spans="5:6" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="E7" s="22" t="s">
+      <c r="E7" s="19" t="s">
         <v>323</v>
       </c>
-      <c r="F7" s="22" t="s">
+      <c r="F7" s="19" t="s">
         <v>324</v>
       </c>
     </row>
     <row r="8" spans="5:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="F8" s="22">
+      <c r="F8" s="19">
         <v>38</v>
       </c>
     </row>
     <row r="9" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E9" s="22" t="s">
+      <c r="E9" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="F9" s="22">
+      <c r="F9" s="19">
         <v>38</v>
       </c>
     </row>
     <row r="10" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E10" s="22" t="s">
+      <c r="E10" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="F10" s="22">
+      <c r="F10" s="19">
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E11" s="22" t="s">
+      <c r="E11" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="F11" s="22">
+      <c r="F11" s="19">
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="5:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="E12" s="22" t="s">
+      <c r="E12" s="19" t="s">
         <v>79</v>
       </c>
-      <c r="F12" s="22">
+      <c r="F12" s="19">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E13" s="22" t="s">
+      <c r="E13" s="19" t="s">
         <v>325</v>
       </c>
-      <c r="F13" s="23">
+      <c r="F13" s="20">
         <v>1</v>
       </c>
     </row>
     <row r="14" spans="5:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="E14" s="22" t="s">
+      <c r="E14" s="19" t="s">
         <v>326</v>
       </c>
-      <c r="F14" s="22" t="s">
+      <c r="F14" s="19" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="15" spans="5:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="E15" s="22" t="s">
+      <c r="E15" s="19" t="s">
         <v>327</v>
       </c>
-      <c r="F15" s="22">
+      <c r="F15" s="19">
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="5:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="E16" s="22" t="s">
+      <c r="E16" s="19" t="s">
         <v>328</v>
       </c>
-      <c r="F16" s="22">
+      <c r="F16" s="19">
         <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="E17" s="22" t="s">
+      <c r="E17" s="19" t="s">
         <v>329</v>
       </c>
-      <c r="F17" s="22" t="s">
+      <c r="F17" s="19" t="s">
         <v>330</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="E18" s="22" t="s">
+      <c r="E18" s="19" t="s">
         <v>331</v>
       </c>
-      <c r="F18" s="22" t="s">
+      <c r="F18" s="19" t="s">
         <v>332</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="35" t="s">
+      <c r="A23" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="B23" s="35" t="s">
+      <c r="B23" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="C23" s="35" t="s">
+      <c r="C23" s="32" t="s">
         <v>76</v>
       </c>
-      <c r="D23" s="35" t="s">
+      <c r="D23" s="32" t="s">
         <v>77</v>
       </c>
-      <c r="E23" s="35" t="s">
+      <c r="E23" s="32" t="s">
         <v>78</v>
       </c>
-      <c r="F23" s="35" t="s">
+      <c r="F23" s="32" t="s">
         <v>325</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="33" t="s">
+      <c r="A24" s="30" t="s">
         <v>74</v>
       </c>
-      <c r="B24" s="33">
+      <c r="B24" s="30">
         <v>8</v>
       </c>
-      <c r="C24" s="33">
+      <c r="C24" s="30">
         <v>8</v>
       </c>
-      <c r="D24" s="33">
+      <c r="D24" s="30">
         <v>0</v>
       </c>
-      <c r="E24" s="33">
+      <c r="E24" s="30">
         <v>0</v>
       </c>
-      <c r="F24" s="34">
+      <c r="F24" s="31">
         <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="33" t="s">
+      <c r="A25" s="30" t="s">
         <v>350</v>
       </c>
-      <c r="B25" s="33">
+      <c r="B25" s="30">
         <v>10</v>
       </c>
-      <c r="C25" s="33">
+      <c r="C25" s="30">
         <v>10</v>
       </c>
-      <c r="D25" s="33">
+      <c r="D25" s="30">
         <v>0</v>
       </c>
-      <c r="E25" s="33">
+      <c r="E25" s="30">
         <v>0</v>
       </c>
-      <c r="F25" s="34">
+      <c r="F25" s="31">
         <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="33" t="s">
+      <c r="A26" s="30" t="s">
         <v>235</v>
       </c>
-      <c r="B26" s="33">
+      <c r="B26" s="30">
         <v>10</v>
       </c>
-      <c r="C26" s="33">
+      <c r="C26" s="30">
         <v>10</v>
       </c>
-      <c r="D26" s="33">
+      <c r="D26" s="30">
         <v>0</v>
       </c>
-      <c r="E26" s="33">
+      <c r="E26" s="30">
         <v>0</v>
       </c>
-      <c r="F26" s="34">
+      <c r="F26" s="31">
         <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="33" t="s">
+      <c r="A27" s="30" t="s">
         <v>296</v>
       </c>
-      <c r="B27" s="33">
+      <c r="B27" s="30">
         <v>10</v>
       </c>
-      <c r="C27" s="33">
+      <c r="C27" s="30">
         <v>10</v>
       </c>
-      <c r="D27" s="33">
+      <c r="D27" s="30">
         <v>0</v>
       </c>
-      <c r="E27" s="33">
+      <c r="E27" s="30">
         <v>0</v>
       </c>
-      <c r="F27" s="34">
+      <c r="F27" s="31">
         <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="33" t="s">
+      <c r="A28" s="30" t="s">
         <v>351</v>
       </c>
-      <c r="B28" s="33">
+      <c r="B28" s="30">
         <v>38</v>
       </c>
-      <c r="C28" s="33">
+      <c r="C28" s="30">
         <v>38</v>
       </c>
-      <c r="D28" s="33">
+      <c r="D28" s="30">
         <v>0</v>
       </c>
-      <c r="E28" s="33">
+      <c r="E28" s="30">
         <v>0</v>
       </c>
-      <c r="F28" s="34">
+      <c r="F28" s="31">
         <v>1</v>
       </c>
     </row>
@@ -2907,388 +2903,388 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="25" t="s">
         <v>333</v>
       </c>
-      <c r="B1" s="28" t="s">
+      <c r="B1" s="25" t="s">
         <v>334</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="10" t="s">
         <v>335</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="10" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="10" t="s">
         <v>336</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="10" t="s">
         <v>337</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="10" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="10" t="s">
         <v>338</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="10" t="s">
         <v>339</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="10" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="10" t="s">
         <v>329</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="10" t="s">
         <v>330</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="10" t="s">
         <v>340</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="10" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="10" t="s">
         <v>341</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="10" t="s">
         <v>324</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="B10" s="11">
+      <c r="B10" s="10">
         <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="10" t="s">
         <v>342</v>
       </c>
-      <c r="B11" s="11">
+      <c r="B11" s="10">
         <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B12" s="11">
+      <c r="B12" s="10">
         <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="B13" s="11">
+      <c r="B13" s="10">
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="B14" s="11">
+      <c r="B14" s="10">
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="B15" s="11">
+      <c r="B15" s="10">
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="10" t="s">
         <v>325</v>
       </c>
-      <c r="B16" s="25">
+      <c r="B16" s="22">
         <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="11" t="s">
+      <c r="A17" s="10" t="s">
         <v>343</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="10" t="s">
         <v>344</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="10" t="s">
         <v>345</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="10" t="s">
         <v>346</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="11" t="s">
+      <c r="A19" s="10" t="s">
         <v>347</v>
       </c>
-      <c r="B19" s="11" t="s">
+      <c r="B19" s="10" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" s="11"/>
-      <c r="B20" s="11"/>
+      <c r="A20" s="10"/>
+      <c r="B20" s="10"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A24" s="28" t="s">
+      <c r="A24" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="B24" s="28" t="s">
+      <c r="B24" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="C24" s="28" t="s">
+      <c r="C24" s="25" t="s">
         <v>348</v>
       </c>
-      <c r="D24" s="28" t="s">
+      <c r="D24" s="25" t="s">
         <v>76</v>
       </c>
-      <c r="E24" s="28" t="s">
+      <c r="E24" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="F24" s="28" t="s">
+      <c r="F24" s="25" t="s">
         <v>78</v>
       </c>
-      <c r="G24" s="28" t="s">
+      <c r="G24" s="25" t="s">
         <v>325</v>
       </c>
-      <c r="H24" s="28" t="s">
+      <c r="H24" s="25" t="s">
         <v>349</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A25" s="26" t="s">
+      <c r="A25" s="23" t="s">
         <v>74</v>
       </c>
-      <c r="B25" s="26">
+      <c r="B25" s="23">
         <v>8</v>
       </c>
-      <c r="C25" s="26">
+      <c r="C25" s="23">
         <v>8</v>
       </c>
-      <c r="D25" s="26">
+      <c r="D25" s="23">
         <v>8</v>
       </c>
-      <c r="E25" s="26">
+      <c r="E25" s="23">
         <v>0</v>
       </c>
-      <c r="F25" s="26">
+      <c r="F25" s="23">
         <v>0</v>
       </c>
-      <c r="G25" s="27">
+      <c r="G25" s="24">
         <v>1</v>
       </c>
-      <c r="H25" s="26" t="s">
+      <c r="H25" s="23" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A26" s="26" t="s">
+      <c r="A26" s="23" t="s">
         <v>350</v>
       </c>
-      <c r="B26" s="26">
+      <c r="B26" s="23">
         <v>10</v>
       </c>
-      <c r="C26" s="26">
+      <c r="C26" s="23">
         <v>10</v>
       </c>
-      <c r="D26" s="26">
+      <c r="D26" s="23">
         <v>10</v>
       </c>
-      <c r="E26" s="26">
+      <c r="E26" s="23">
         <v>0</v>
       </c>
-      <c r="F26" s="26">
+      <c r="F26" s="23">
         <v>0</v>
       </c>
-      <c r="G26" s="27">
+      <c r="G26" s="24">
         <v>1</v>
       </c>
-      <c r="H26" s="26" t="s">
+      <c r="H26" s="23" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A27" s="26" t="s">
+      <c r="A27" s="23" t="s">
         <v>235</v>
       </c>
-      <c r="B27" s="26">
+      <c r="B27" s="23">
         <v>10</v>
       </c>
-      <c r="C27" s="26">
+      <c r="C27" s="23">
         <v>10</v>
       </c>
-      <c r="D27" s="26">
+      <c r="D27" s="23">
         <v>10</v>
       </c>
-      <c r="E27" s="26">
+      <c r="E27" s="23">
         <v>0</v>
       </c>
-      <c r="F27" s="26">
+      <c r="F27" s="23">
         <v>0</v>
       </c>
-      <c r="G27" s="27">
+      <c r="G27" s="24">
         <v>1</v>
       </c>
-      <c r="H27" s="26" t="s">
+      <c r="H27" s="23" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A28" s="26" t="s">
+      <c r="A28" s="23" t="s">
         <v>296</v>
       </c>
-      <c r="B28" s="26">
+      <c r="B28" s="23">
         <v>10</v>
       </c>
-      <c r="C28" s="26">
+      <c r="C28" s="23">
         <v>10</v>
       </c>
-      <c r="D28" s="26">
+      <c r="D28" s="23">
         <v>10</v>
       </c>
-      <c r="E28" s="26">
+      <c r="E28" s="23">
         <v>0</v>
       </c>
-      <c r="F28" s="26">
+      <c r="F28" s="23">
         <v>0</v>
       </c>
-      <c r="G28" s="27">
+      <c r="G28" s="24">
         <v>1</v>
       </c>
-      <c r="H28" s="26" t="s">
+      <c r="H28" s="23" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A29" s="26" t="s">
+      <c r="A29" s="23" t="s">
         <v>351</v>
       </c>
-      <c r="B29" s="26">
+      <c r="B29" s="23">
         <v>38</v>
       </c>
-      <c r="C29" s="26">
+      <c r="C29" s="23">
         <v>38</v>
       </c>
-      <c r="D29" s="26">
+      <c r="D29" s="23">
         <v>38</v>
       </c>
-      <c r="E29" s="26">
+      <c r="E29" s="23">
         <v>0</v>
       </c>
-      <c r="F29" s="26">
+      <c r="F29" s="23">
         <v>0</v>
       </c>
-      <c r="G29" s="27">
+      <c r="G29" s="24">
         <v>1</v>
       </c>
-      <c r="H29" s="26" t="s">
+      <c r="H29" s="23" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="30" t="s">
+      <c r="A35" s="27" t="s">
         <v>69</v>
       </c>
-      <c r="B35" s="30" t="s">
+      <c r="B35" s="27" t="s">
         <v>334</v>
       </c>
-      <c r="C35" s="29"/>
-      <c r="D35" s="29"/>
-      <c r="E35" s="29"/>
-      <c r="F35" s="29"/>
+      <c r="C35" s="26"/>
+      <c r="D35" s="26"/>
+      <c r="E35" s="26"/>
+      <c r="F35" s="26"/>
     </row>
     <row r="36" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A36" s="31" t="s">
+      <c r="A36" s="28" t="s">
         <v>352</v>
       </c>
-      <c r="B36" s="32" t="s">
+      <c r="B36" s="29" t="s">
         <v>353</v>
       </c>
-      <c r="C36" s="31"/>
-      <c r="D36" s="31"/>
-      <c r="E36" s="31"/>
-      <c r="F36" s="31"/>
+      <c r="C36" s="28"/>
+      <c r="D36" s="28"/>
+      <c r="E36" s="28"/>
+      <c r="F36" s="28"/>
     </row>
     <row r="37" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A37" s="31" t="s">
+      <c r="A37" s="28" t="s">
         <v>354</v>
       </c>
-      <c r="B37" s="32" t="s">
+      <c r="B37" s="29" t="s">
         <v>355</v>
       </c>
-      <c r="C37" s="31"/>
-      <c r="D37" s="31"/>
-      <c r="E37" s="31"/>
-      <c r="F37" s="31"/>
+      <c r="C37" s="28"/>
+      <c r="D37" s="28"/>
+      <c r="E37" s="28"/>
+      <c r="F37" s="28"/>
     </row>
     <row r="38" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A38" s="31" t="s">
+      <c r="A38" s="28" t="s">
         <v>356</v>
       </c>
-      <c r="B38" s="32" t="s">
+      <c r="B38" s="29" t="s">
         <v>357</v>
       </c>
-      <c r="C38" s="31"/>
-      <c r="D38" s="31"/>
-      <c r="E38" s="31"/>
-      <c r="F38" s="31"/>
+      <c r="C38" s="28"/>
+      <c r="D38" s="28"/>
+      <c r="E38" s="28"/>
+      <c r="F38" s="28"/>
     </row>
     <row r="39" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A39" s="31" t="s">
+      <c r="A39" s="28" t="s">
         <v>358</v>
       </c>
-      <c r="B39" s="32" t="s">
+      <c r="B39" s="29" t="s">
         <v>359</v>
       </c>
-      <c r="C39" s="31"/>
-      <c r="D39" s="31"/>
-      <c r="E39" s="31"/>
-      <c r="F39" s="31"/>
+      <c r="C39" s="28"/>
+      <c r="D39" s="28"/>
+      <c r="E39" s="28"/>
+      <c r="F39" s="28"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="31" t="s">
+      <c r="A40" s="28" t="s">
         <v>360</v>
       </c>
-      <c r="B40" s="31" t="s">
+      <c r="B40" s="28" t="s">
         <v>34</v>
       </c>
-      <c r="C40" s="31"/>
-      <c r="D40" s="31"/>
-      <c r="E40" s="31"/>
-      <c r="F40" s="31"/>
+      <c r="C40" s="28"/>
+      <c r="D40" s="28"/>
+      <c r="E40" s="28"/>
+      <c r="F40" s="28"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3305,10 +3301,10 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="8" t="s">
         <v>70</v>
       </c>
     </row>
@@ -3412,31 +3408,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="10" t="s">
         <v>24</v>
       </c>
     </row>
@@ -3455,7 +3451,7 @@
       <c r="A3" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>86</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -3470,7 +3466,7 @@
       <c r="F3" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="3" t="s">
         <v>32</v>
       </c>
       <c r="H3" s="2" t="s">
@@ -3536,7 +3532,7 @@
       <c r="A8" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>90</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -3548,10 +3544,10 @@
       <c r="E8" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="3" t="s">
         <v>96</v>
       </c>
       <c r="H8" s="2" t="s">
@@ -3615,7 +3611,7 @@
       <c r="A13" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>98</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -3627,10 +3623,10 @@
       <c r="E13" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="F13" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="G13" s="3" t="s">
         <v>105</v>
       </c>
       <c r="H13" s="2" t="s">
@@ -3681,7 +3677,7 @@
       <c r="A17" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="3" t="s">
         <v>107</v>
       </c>
       <c r="C17" s="2" t="s">
@@ -3696,7 +3692,7 @@
       <c r="F17" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="G17" s="4" t="s">
+      <c r="G17" s="3" t="s">
         <v>112</v>
       </c>
       <c r="H17" s="2" t="s">
@@ -3758,7 +3754,7 @@
       <c r="A22" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="3" t="s">
         <v>114</v>
       </c>
       <c r="C22" s="2" t="s">
@@ -3770,10 +3766,10 @@
       <c r="E22" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="F22" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="G22" s="4" t="s">
+      <c r="G22" s="3" t="s">
         <v>119</v>
       </c>
       <c r="H22" s="2" t="s">
@@ -3835,22 +3831,22 @@
       <c r="A27" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="3" t="s">
         <v>121</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="D27" s="12" t="s">
+      <c r="D27" s="11" t="s">
         <v>100</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="F27" s="4" t="s">
+      <c r="F27" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="G27" s="4" t="s">
+      <c r="G27" s="3" t="s">
         <v>128</v>
       </c>
       <c r="H27" s="2" t="s">
@@ -3938,7 +3934,7 @@
       <c r="A34" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="B34" s="4" t="s">
+      <c r="B34" s="3" t="s">
         <v>130</v>
       </c>
       <c r="C34" s="2" t="s">
@@ -3950,10 +3946,10 @@
       <c r="E34" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="F34" s="4" t="s">
+      <c r="F34" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="G34" s="4" t="s">
+      <c r="G34" s="3" t="s">
         <v>136</v>
       </c>
       <c r="H34" s="2" t="s">
@@ -4030,7 +4026,7 @@
       <c r="A40" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="B40" s="4" t="s">
+      <c r="B40" s="3" t="s">
         <v>138</v>
       </c>
       <c r="C40" s="2" t="s">
@@ -4039,19 +4035,19 @@
       <c r="D40" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E40" s="4" t="s">
+      <c r="E40" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="F40" s="4" t="s">
+      <c r="F40" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="G40" s="4" t="s">
+      <c r="G40" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="H40" s="4" t="s">
+      <c r="H40" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="I40" s="4" t="s">
+      <c r="I40" s="3" t="s">
         <v>35</v>
       </c>
     </row>
@@ -4109,7 +4105,7 @@
       <c r="A45" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="B45" s="4" t="s">
+      <c r="B45" s="3" t="s">
         <v>146</v>
       </c>
       <c r="C45" s="2" t="s">
@@ -4118,19 +4114,19 @@
       <c r="D45" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E45" s="4" t="s">
+      <c r="E45" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="F45" s="4" t="s">
+      <c r="F45" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="G45" s="4" t="s">
+      <c r="G45" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="H45" s="4" t="s">
+      <c r="H45" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="I45" s="4" t="s">
+      <c r="I45" s="3" t="s">
         <v>35</v>
       </c>
     </row>
@@ -4199,26 +4195,26 @@
       <c r="A51" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="B51" s="4" t="s">
+      <c r="B51" s="3" t="s">
         <v>153</v>
       </c>
       <c r="C51" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="D51" s="13"/>
-      <c r="E51" s="4" t="s">
+      <c r="D51" s="12"/>
+      <c r="E51" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="F51" s="4" t="s">
+      <c r="F51" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="G51" s="4" t="s">
+      <c r="G51" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="H51" s="4" t="s">
+      <c r="H51" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="I51" s="4" t="s">
+      <c r="I51" s="3" t="s">
         <v>35</v>
       </c>
     </row>
@@ -4226,7 +4222,7 @@
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
-      <c r="D52" s="14" t="s">
+      <c r="D52" s="11" t="s">
         <v>100</v>
       </c>
       <c r="E52" s="2"/>
@@ -4329,31 +4325,31 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="G2" s="15" t="s">
+      <c r="G2" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="H2" s="15" t="s">
+      <c r="H2" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="I2" s="15" t="s">
+      <c r="I2" s="13" t="s">
         <v>24</v>
       </c>
       <c r="J2" s="2"/>
@@ -4374,7 +4370,7 @@
       <c r="A4" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>163</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -4386,10 +4382,10 @@
       <c r="E4" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="3" t="s">
         <v>225</v>
       </c>
       <c r="H4" s="2" t="s">
@@ -4444,7 +4440,7 @@
       <c r="A8" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>169</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -4456,10 +4452,10 @@
       <c r="E8" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="3" t="s">
         <v>226</v>
       </c>
       <c r="H8" s="2" t="s">
@@ -4526,7 +4522,7 @@
       <c r="A13" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>176</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -4538,10 +4534,10 @@
       <c r="E13" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="F13" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="G13" s="3" t="s">
         <v>227</v>
       </c>
       <c r="H13" s="2" t="s">
@@ -4610,20 +4606,20 @@
       <c r="A18" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="3" t="s">
         <v>183</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="D18" s="14"/>
+      <c r="D18" s="11"/>
       <c r="E18" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="F18" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="G18" s="4" t="s">
+      <c r="G18" s="3" t="s">
         <v>228</v>
       </c>
       <c r="H18" s="2" t="s">
@@ -4638,7 +4634,7 @@
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
-      <c r="D19" s="14" t="s">
+      <c r="D19" s="11" t="s">
         <v>171</v>
       </c>
       <c r="E19" s="2"/>
@@ -4652,7 +4648,7 @@
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
-      <c r="D20" s="14" t="s">
+      <c r="D20" s="11" t="s">
         <v>178</v>
       </c>
       <c r="E20" s="2"/>
@@ -4666,7 +4662,7 @@
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
-      <c r="D21" s="14" t="s">
+      <c r="D21" s="11" t="s">
         <v>179</v>
       </c>
       <c r="E21" s="2"/>
@@ -4680,7 +4676,7 @@
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
-      <c r="D22" s="14" t="s">
+      <c r="D22" s="11" t="s">
         <v>185</v>
       </c>
       <c r="E22" s="2"/>
@@ -4706,7 +4702,7 @@
       <c r="A24" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="3" t="s">
         <v>188</v>
       </c>
       <c r="C24" s="2" t="s">
@@ -4718,10 +4714,10 @@
       <c r="E24" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="F24" s="4" t="s">
+      <c r="F24" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="G24" s="4" t="s">
+      <c r="G24" s="3" t="s">
         <v>229</v>
       </c>
       <c r="H24" s="2" t="s">
@@ -4802,20 +4798,20 @@
       <c r="A30" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="B30" s="3" t="s">
         <v>146</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="D30" s="14"/>
+      <c r="D30" s="11"/>
       <c r="E30" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="F30" s="4" t="s">
+      <c r="F30" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="G30" s="4" t="s">
+      <c r="G30" s="3" t="s">
         <v>230</v>
       </c>
       <c r="H30" s="2" t="s">
@@ -4830,7 +4826,7 @@
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
-      <c r="D31" s="14" t="s">
+      <c r="D31" s="11" t="s">
         <v>171</v>
       </c>
       <c r="E31" s="2"/>
@@ -4844,7 +4840,7 @@
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
-      <c r="D32" s="14" t="s">
+      <c r="D32" s="11" t="s">
         <v>178</v>
       </c>
       <c r="E32" s="2"/>
@@ -4858,7 +4854,7 @@
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
-      <c r="D33" s="14" t="s">
+      <c r="D33" s="11" t="s">
         <v>179</v>
       </c>
       <c r="E33" s="2"/>
@@ -4872,7 +4868,7 @@
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
-      <c r="D34" s="14" t="s">
+      <c r="D34" s="11" t="s">
         <v>196</v>
       </c>
       <c r="E34" s="2"/>
@@ -4910,7 +4906,7 @@
       <c r="A37" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="B37" s="4" t="s">
+      <c r="B37" s="3" t="s">
         <v>153</v>
       </c>
       <c r="C37" s="2" t="s">
@@ -4922,10 +4918,10 @@
       <c r="E37" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="F37" s="4" t="s">
+      <c r="F37" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="G37" s="4" t="s">
+      <c r="G37" s="3" t="s">
         <v>161</v>
       </c>
       <c r="H37" s="2" t="s">
@@ -5020,7 +5016,7 @@
       <c r="A44" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="B44" s="4" t="s">
+      <c r="B44" s="3" t="s">
         <v>207</v>
       </c>
       <c r="C44" s="2" t="s">
@@ -5032,10 +5028,10 @@
       <c r="E44" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="F44" s="4" t="s">
+      <c r="F44" s="3" t="s">
         <v>213</v>
       </c>
-      <c r="G44" s="4" t="s">
+      <c r="G44" s="3" t="s">
         <v>231</v>
       </c>
       <c r="H44" s="2" t="s">
@@ -5118,7 +5114,7 @@
       <c r="A50" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="B50" s="4" t="s">
+      <c r="B50" s="3" t="s">
         <v>215</v>
       </c>
       <c r="C50" s="2" t="s">
@@ -5130,10 +5126,10 @@
       <c r="E50" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="F50" s="4" t="s">
+      <c r="F50" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="G50" s="4" t="s">
+      <c r="G50" s="3" t="s">
         <v>232</v>
       </c>
       <c r="H50" s="2" t="s">
@@ -5214,20 +5210,20 @@
       <c r="A56" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="B56" s="4" t="s">
+      <c r="B56" s="3" t="s">
         <v>221</v>
       </c>
       <c r="C56" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="D56" s="14"/>
+      <c r="D56" s="11"/>
       <c r="E56" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="F56" s="4" t="s">
+      <c r="F56" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="G56" s="4" t="s">
+      <c r="G56" s="3" t="s">
         <v>233</v>
       </c>
       <c r="H56" s="2" t="s">
@@ -5242,7 +5238,7 @@
       <c r="A57" s="2"/>
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
-      <c r="D57" s="14" t="s">
+      <c r="D57" s="11" t="s">
         <v>171</v>
       </c>
       <c r="E57" s="2"/>
@@ -5256,7 +5252,7 @@
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
-      <c r="D58" s="14" t="s">
+      <c r="D58" s="11" t="s">
         <v>217</v>
       </c>
       <c r="E58" s="2"/>
@@ -5270,7 +5266,7 @@
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
-      <c r="D59" s="14" t="s">
+      <c r="D59" s="11" t="s">
         <v>179</v>
       </c>
       <c r="E59" s="2"/>
@@ -5284,7 +5280,7 @@
       <c r="A60" s="2"/>
       <c r="B60" s="2"/>
       <c r="C60" s="2"/>
-      <c r="D60" s="14" t="s">
+      <c r="D60" s="11" t="s">
         <v>223</v>
       </c>
       <c r="E60" s="2"/>
@@ -5347,90 +5343,90 @@
   </cols>
   <sheetData>
     <row r="2" spans="3:4" x14ac:dyDescent="0.3">
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="15" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="3" spans="3:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="16" t="s">
+      <c r="D3" s="14" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="4" spans="3:4" x14ac:dyDescent="0.3">
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="D4" s="14" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="5" spans="3:4" x14ac:dyDescent="0.3">
-      <c r="C5" s="16" t="s">
+      <c r="C5" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="D5" s="16">
+      <c r="D5" s="14">
         <v>10</v>
       </c>
     </row>
     <row r="6" spans="3:4" x14ac:dyDescent="0.3">
-      <c r="C6" s="16" t="s">
+      <c r="C6" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="D6" s="16">
+      <c r="D6" s="14">
         <v>10</v>
       </c>
     </row>
     <row r="7" spans="3:4" x14ac:dyDescent="0.3">
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="14">
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="3:4" x14ac:dyDescent="0.3">
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="D8" s="16">
+      <c r="D8" s="14">
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="3:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="D9" s="16">
+      <c r="D9" s="14">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="3:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C10" s="16" t="s">
+      <c r="C10" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="D10" s="16" t="s">
+      <c r="D10" s="14" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="11" spans="3:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="D11" s="16" t="s">
+      <c r="D11" s="14" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="12" spans="3:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C12" s="16" t="s">
+      <c r="C12" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="D12" s="16" t="s">
+      <c r="D12" s="14" t="s">
         <v>84</v>
       </c>
     </row>
@@ -5455,373 +5451,373 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="E1" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="18" t="s">
+      <c r="F1" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="18" t="s">
+      <c r="G1" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="18" t="s">
+      <c r="H1" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="18" t="s">
+      <c r="I1" s="16" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="11" t="s">
         <v>236</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="11" t="s">
         <v>237</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="11" t="s">
         <v>238</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="D2" s="11" t="s">
         <v>316</v>
       </c>
-      <c r="E2" s="14" t="s">
+      <c r="E2" s="11" t="s">
         <v>295</v>
       </c>
-      <c r="F2" s="14" t="s">
+      <c r="F2" s="11" t="s">
         <v>239</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="G2" s="11" t="s">
         <v>240</v>
       </c>
-      <c r="H2" s="14" t="s">
+      <c r="H2" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="I2" s="14" t="s">
+      <c r="I2" s="11" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="11" t="s">
         <v>241</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="11" t="s">
         <v>242</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="11" t="s">
         <v>243</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" s="11" t="s">
         <v>317</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="E3" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="F3" s="11" t="s">
         <v>244</v>
       </c>
-      <c r="G3" s="14" t="s">
+      <c r="G3" s="11" t="s">
         <v>245</v>
       </c>
-      <c r="H3" s="14" t="s">
+      <c r="H3" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="I3" s="14" t="s">
+      <c r="I3" s="11" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="11" t="s">
         <v>246</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="11" t="s">
         <v>247</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="11" t="s">
         <v>248</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="11" t="s">
         <v>318</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="E4" s="11" t="s">
         <v>249</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="11" t="s">
         <v>250</v>
       </c>
-      <c r="G4" s="14" t="s">
+      <c r="G4" s="11" t="s">
         <v>251</v>
       </c>
-      <c r="H4" s="14" t="s">
+      <c r="H4" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="I4" s="14" t="s">
+      <c r="I4" s="11" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="33" t="s">
         <v>252</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="33" t="s">
         <v>253</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="33" t="s">
         <v>254</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="33" t="s">
         <v>321</v>
       </c>
-      <c r="E5" s="14" t="s">
+      <c r="E5" s="11" t="s">
         <v>255</v>
       </c>
-      <c r="F5" s="19" t="s">
+      <c r="F5" s="33" t="s">
         <v>258</v>
       </c>
-      <c r="G5" s="19" t="s">
+      <c r="G5" s="33" t="s">
         <v>259</v>
       </c>
-      <c r="H5" s="19" t="s">
+      <c r="H5" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="I5" s="19" t="s">
+      <c r="I5" s="33" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="19"/>
-      <c r="B6" s="19"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="14" t="s">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" s="33"/>
+      <c r="B6" s="33"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="11" t="s">
         <v>256</v>
       </c>
-      <c r="F6" s="19"/>
-      <c r="G6" s="19"/>
-      <c r="H6" s="19"/>
-      <c r="I6" s="19"/>
-    </row>
-    <row r="7" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="19"/>
-      <c r="B7" s="19"/>
-      <c r="C7" s="19"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="14" t="s">
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="33"/>
+      <c r="I6" s="33"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" s="33"/>
+      <c r="B7" s="33"/>
+      <c r="C7" s="33"/>
+      <c r="D7" s="33"/>
+      <c r="E7" s="11" t="s">
         <v>257</v>
       </c>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19"/>
-      <c r="I7" s="19"/>
+      <c r="F7" s="33"/>
+      <c r="G7" s="33"/>
+      <c r="H7" s="33"/>
+      <c r="I7" s="33"/>
     </row>
     <row r="8" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="33" t="s">
         <v>260</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="33" t="s">
         <v>261</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="33" t="s">
         <v>262</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="33" t="s">
         <v>313</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="11" t="s">
         <v>263</v>
       </c>
-      <c r="F8" s="19" t="s">
+      <c r="F8" s="33" t="s">
         <v>265</v>
       </c>
-      <c r="G8" s="19" t="s">
+      <c r="G8" s="33" t="s">
         <v>266</v>
       </c>
-      <c r="H8" s="19" t="s">
+      <c r="H8" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="I8" s="19" t="s">
+      <c r="I8" s="33" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A9" s="19"/>
-      <c r="B9" s="19"/>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="14" t="s">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" s="33"/>
+      <c r="B9" s="33"/>
+      <c r="C9" s="33"/>
+      <c r="D9" s="33"/>
+      <c r="E9" s="11" t="s">
         <v>264</v>
       </c>
-      <c r="F9" s="19"/>
-      <c r="G9" s="19"/>
-      <c r="H9" s="19"/>
-      <c r="I9" s="19"/>
-    </row>
-    <row r="10" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="19"/>
-      <c r="B10" s="19"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="14" t="s">
+      <c r="F9" s="33"/>
+      <c r="G9" s="33"/>
+      <c r="H9" s="33"/>
+      <c r="I9" s="33"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A10" s="33"/>
+      <c r="B10" s="33"/>
+      <c r="C10" s="33"/>
+      <c r="D10" s="33"/>
+      <c r="E10" s="11" t="s">
         <v>257</v>
       </c>
-      <c r="F10" s="19"/>
-      <c r="G10" s="19"/>
-      <c r="H10" s="19"/>
-      <c r="I10" s="19"/>
+      <c r="F10" s="33"/>
+      <c r="G10" s="33"/>
+      <c r="H10" s="33"/>
+      <c r="I10" s="33"/>
     </row>
     <row r="11" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="11" t="s">
         <v>267</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="11" t="s">
         <v>268</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="11" t="s">
         <v>269</v>
       </c>
-      <c r="D11" s="14" t="s">
+      <c r="D11" s="11" t="s">
         <v>314</v>
       </c>
-      <c r="E11" s="14" t="s">
+      <c r="E11" s="11" t="s">
         <v>270</v>
       </c>
-      <c r="F11" s="14" t="s">
+      <c r="F11" s="11" t="s">
         <v>271</v>
       </c>
-      <c r="G11" s="14" t="s">
+      <c r="G11" s="11" t="s">
         <v>272</v>
       </c>
-      <c r="H11" s="14" t="s">
+      <c r="H11" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="I11" s="14" t="s">
+      <c r="I11" s="11" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="72" x14ac:dyDescent="0.3">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="11" t="s">
         <v>273</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="11" t="s">
         <v>274</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="11" t="s">
         <v>275</v>
       </c>
-      <c r="D12" s="14" t="s">
+      <c r="D12" s="11" t="s">
         <v>315</v>
       </c>
-      <c r="E12" s="14" t="s">
+      <c r="E12" s="11" t="s">
         <v>276</v>
       </c>
-      <c r="F12" s="14" t="s">
+      <c r="F12" s="11" t="s">
         <v>277</v>
       </c>
-      <c r="G12" s="14" t="s">
+      <c r="G12" s="11" t="s">
         <v>278</v>
       </c>
-      <c r="H12" s="14" t="s">
+      <c r="H12" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="I12" s="14" t="s">
+      <c r="I12" s="11" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="11" t="s">
         <v>279</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="B13" s="11" t="s">
         <v>280</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="C13" s="11" t="s">
         <v>281</v>
       </c>
-      <c r="D13" s="14" t="s">
+      <c r="D13" s="11" t="s">
         <v>319</v>
       </c>
-      <c r="E13" s="14" t="s">
+      <c r="E13" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="F13" s="14" t="s">
+      <c r="F13" s="11" t="s">
         <v>282</v>
       </c>
-      <c r="G13" s="14" t="s">
+      <c r="G13" s="11" t="s">
         <v>283</v>
       </c>
-      <c r="H13" s="14" t="s">
+      <c r="H13" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="I13" s="14" t="s">
+      <c r="I13" s="11" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A14" s="14" t="s">
+      <c r="A14" s="11" t="s">
         <v>284</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="11" t="s">
         <v>285</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="C14" s="11" t="s">
         <v>286</v>
       </c>
-      <c r="D14" s="14" t="s">
+      <c r="D14" s="11" t="s">
         <v>320</v>
       </c>
-      <c r="E14" s="14" t="s">
+      <c r="E14" s="11" t="s">
         <v>287</v>
       </c>
-      <c r="F14" s="14" t="s">
+      <c r="F14" s="11" t="s">
         <v>288</v>
       </c>
-      <c r="G14" s="14" t="s">
+      <c r="G14" s="11" t="s">
         <v>289</v>
       </c>
-      <c r="H14" s="14" t="s">
+      <c r="H14" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="I14" s="14" t="s">
+      <c r="I14" s="11" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="72" x14ac:dyDescent="0.3">
-      <c r="A15" s="14" t="s">
+      <c r="A15" s="11" t="s">
         <v>290</v>
       </c>
-      <c r="B15" s="14" t="s">
+      <c r="B15" s="11" t="s">
         <v>291</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="C15" s="11" t="s">
         <v>292</v>
       </c>
-      <c r="D15" s="14" t="s">
+      <c r="D15" s="11" t="s">
         <v>322</v>
       </c>
-      <c r="E15" s="14" t="s">
+      <c r="E15" s="11" t="s">
         <v>249</v>
       </c>
-      <c r="F15" s="14" t="s">
+      <c r="F15" s="11" t="s">
         <v>293</v>
       </c>
-      <c r="G15" s="14" t="s">
+      <c r="G15" s="11" t="s">
         <v>294</v>
       </c>
-      <c r="H15" s="14" t="s">
+      <c r="H15" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="I15" s="14" t="s">
+      <c r="I15" s="11" t="s">
         <v>35</v>
       </c>
     </row>
@@ -5860,90 +5856,90 @@
   </cols>
   <sheetData>
     <row r="2" spans="6:7" x14ac:dyDescent="0.3">
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="18" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="3" spans="6:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="F3" s="20" t="s">
+      <c r="F3" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="G3" s="20" t="s">
+      <c r="G3" s="17" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="4" spans="6:7" x14ac:dyDescent="0.3">
-      <c r="F4" s="20" t="s">
+      <c r="F4" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="G4" s="20" t="s">
+      <c r="G4" s="17" t="s">
         <v>296</v>
       </c>
     </row>
     <row r="5" spans="6:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="F5" s="20" t="s">
+      <c r="F5" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="G5" s="20">
+      <c r="G5" s="17">
         <v>10</v>
       </c>
     </row>
     <row r="6" spans="6:7" x14ac:dyDescent="0.3">
-      <c r="F6" s="20" t="s">
+      <c r="F6" s="17" t="s">
         <v>76</v>
       </c>
-      <c r="G6" s="20">
+      <c r="G6" s="17">
         <v>10</v>
       </c>
     </row>
     <row r="7" spans="6:7" x14ac:dyDescent="0.3">
-      <c r="F7" s="20" t="s">
+      <c r="F7" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="G7" s="20">
+      <c r="G7" s="17">
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="6:7" x14ac:dyDescent="0.3">
-      <c r="F8" s="20" t="s">
+      <c r="F8" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="G8" s="20">
+      <c r="G8" s="17">
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="6:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="F9" s="20" t="s">
+      <c r="F9" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="G9" s="20">
+      <c r="G9" s="17">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="6:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="F10" s="20" t="s">
+      <c r="F10" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="G10" s="20" t="s">
+      <c r="G10" s="17" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="11" spans="6:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="F11" s="20" t="s">
+      <c r="F11" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="G11" s="20" t="s">
+      <c r="G11" s="17" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="12" spans="6:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="F12" s="20" t="s">
+      <c r="F12" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="G12" s="20" t="s">
+      <c r="G12" s="17" t="s">
         <v>84</v>
       </c>
     </row>

</xml_diff>